<commit_message>
Stop two remark cells being parsed as formulas
The dosage and cost rows carried explanatory notes in the remark column
that began with "=", which Excel reads as a formula and renders as
#NAME?. Reworded both to plain text.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UEsLPMwF69aavPNwWVFuSY
</commit_message>
<xml_diff>
--- a/Unitor_연료유첨가제_제품자료_3종.xlsx
+++ b/Unitor_연료유첨가제_제품자료_3종.xlsx
@@ -1335,9 +1335,10 @@
         <f>ROUND(1000/E21,0)</f>
         <v/>
       </c>
-      <c r="F22" s="7">
-        <f> ROUND(1000 / 처리톤수, 0)</f>
-        <v/>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>1,000 ÷ 처리톤수 (자동 계산)</t>
+        </is>
       </c>
     </row>
     <row r="23" ht="46" customHeight="1">
@@ -1375,9 +1376,10 @@
         <f>IF(E23="","",E22*E23)</f>
         <v/>
       </c>
-      <c r="F24" s="7">
-        <f> 투입량 × 단가 (자동 계산)</f>
-        <v/>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>투입량 × 단가 (자동 계산)</t>
+        </is>
       </c>
     </row>
     <row r="25" ht="46" customHeight="1">

</xml_diff>

<commit_message>
Align dosage basis on 100 ppm and drop the fuel-grade matrix sheet
Catalyst now leads with "약 1.5%" fuel saving, carrying the measured
1.454% (VLSFO) alongside it, and its general dosage moves from 1L:15MT to
1L:10MT so the quoted saving and the quoted volume come from the same
test condition. The product-spec 1L:15MT stays available as its own row
on the calculation sheet.

DieselPower Lubricity keeps only the 100 ppm result (535 -> 396 µm); the
150 ppm / 355 µm row is gone, as is its 125 ppm calculation row.

The fuel-grade matrix sheet is removed at the customer's request — the
per-product fuel coverage still appears in the summary sheet's 적용 유종
row.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UEsLPMwF69aavPNwWVFuSY
</commit_message>
<xml_diff>
--- a/Unitor_연료유첨가제_제품자료_3종.xlsx
+++ b/Unitor_연료유첨가제_제품자료_3종.xlsx
@@ -8,9 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="제품 요약" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="유종별 적용" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Reference 상세" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="투입량·비용 산출" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Reference 상세" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="투입량·비용 산출" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -28,7 +27,7 @@
     <numFmt numFmtId="169" formatCode="0&quot;℃&quot;"/>
     <numFmt numFmtId="170" formatCode="#,##0&quot;  MT&quot;"/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="20">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -84,14 +83,14 @@
     <font>
       <name val="맑은 고딕"/>
       <b val="1"/>
-      <color rgb="00C00000"/>
-      <sz val="9"/>
+      <color rgb="000000FF"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="맑은 고딕"/>
       <b val="1"/>
-      <color rgb="000000FF"/>
-      <sz val="10"/>
+      <color rgb="00C00000"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="맑은 고딕"/>
@@ -104,24 +103,6 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="14"/>
-    </font>
-    <font>
-      <name val="맑은 고딕"/>
-      <b val="1"/>
-      <color rgb="001F3864"/>
-      <sz val="13"/>
-    </font>
-    <font>
-      <name val="맑은 고딕"/>
-      <b val="1"/>
-      <color rgb="00A6A6A6"/>
-      <sz val="13"/>
-    </font>
-    <font>
-      <name val="맑은 고딕"/>
-      <b val="1"/>
-      <color rgb="00BF8F00"/>
-      <sz val="13"/>
     </font>
     <font>
       <name val="맑은 고딕"/>
@@ -266,7 +247,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -299,17 +280,17 @@
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="167" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -320,80 +301,68 @@
     <xf numFmtId="0" fontId="12" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="14" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="19" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="17" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="22" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -784,7 +753,7 @@
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>※ 고객 요청 양식 기준 재구성 · 제품 3종 (FuelPower Conditioner / FuelPower Catalyst / DieselPower Lubricity)
-※ 제품별 적용 유종이 상이하여 열(column)을 「유종」이 아닌 「제품」 기준으로 배열하고, 유종 적용 범위는 별도 행 및 '유종별 적용' 시트에 표기</t>
+※ 제품별 적용 유종이 상이하여 열(column)을 「유종」이 아닌 「제품」 기준으로 배열하고, 유종 적용 범위는 '적용 유종' 행에 표기</t>
         </is>
       </c>
     </row>
@@ -964,7 +933,8 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>상세: '유종별 적용' 시트 참조</t>
+          <t>Conditioner · Catalyst 는 잔사유,
+Lubricity 는 증류유 전용</t>
         </is>
       </c>
     </row>
@@ -1187,8 +1157,8 @@
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>1L : 15 MT
-(1 : 15,000)</t>
+          <t>1L : 10 MT
+(1 : 10,000, 100 ppm)</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
@@ -1266,26 +1236,28 @@
       <c r="C20" s="9" t="inlineStr">
         <is>
           <t>Hot Spin 시험 기준
-(제품 자료상 1 : 10,000 적용 사례 있음)</t>
+(Catalyst 병용 실선 시험은
+1L : 10 MT 조건)</t>
         </is>
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
           <t>100 ppm = 1L : 10 MT
-★ SFOC 개선 실측 데이터는 전부
-100 ppm 조건에서 취득</t>
+→ SFOC 개선 실측 데이터
+   전부 이 조건에서 취득</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
-          <t>125 ppm = 0.125 L/ton
-→ HFRR 460 µm 미만 달성</t>
-        </is>
-      </c>
-      <c r="F20" s="12" t="inlineStr">
-        <is>
-          <t>★ 연료절감을 목적으로 할 경우
-Catalyst는 1L : 10 MT 적용 권장</t>
+          <t>100 ppm = 1L : 10 MT
+→ HFRR 396 µm 달성</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>3개 제품 모두 100 ppm(1L : 10 MT)
+기준으로 정리 (Conditioner 는
+제품 사양상 General 1L : 15 MT)</t>
         </is>
       </c>
     </row>
@@ -1301,13 +1273,13 @@
 (1 L 당 처리 톤수, MT)</t>
         </is>
       </c>
-      <c r="C21" s="13" t="n">
+      <c r="C21" s="12" t="n">
         <v>15</v>
       </c>
-      <c r="D21" s="13" t="n">
-        <v>15</v>
-      </c>
-      <c r="E21" s="13" t="n">
+      <c r="D21" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="E21" s="12" t="n">
         <v>10</v>
       </c>
       <c r="F21" s="7" t="inlineStr">
@@ -1323,15 +1295,15 @@
           <t>1,000 M/T 기준 투입량 (L)</t>
         </is>
       </c>
-      <c r="C22" s="14">
+      <c r="C22" s="13">
         <f>ROUND(1000/C21,0)</f>
         <v/>
       </c>
-      <c r="D22" s="14">
+      <c r="D22" s="13">
         <f>ROUND(1000/D21,0)</f>
         <v/>
       </c>
-      <c r="E22" s="14">
+      <c r="E22" s="13">
         <f>ROUND(1000/E21,0)</f>
         <v/>
       </c>
@@ -1348,10 +1320,10 @@
           <t>제품단가 (USD / LITER)</t>
         </is>
       </c>
-      <c r="C23" s="15" t="n"/>
-      <c r="D23" s="15" t="n"/>
-      <c r="E23" s="15" t="n"/>
-      <c r="F23" s="12" t="inlineStr">
+      <c r="C23" s="14" t="n"/>
+      <c r="D23" s="14" t="n"/>
+      <c r="E23" s="14" t="n"/>
+      <c r="F23" s="15" t="inlineStr">
         <is>
           <t>★ 노란색 셀에 단가 입력</t>
         </is>
@@ -1484,15 +1456,16 @@
       <c r="C28" s="9" t="inlineStr">
         <is>
           <t>단독 기준 연료절감률 미제시
-(보증 불가)
 ※ Catalyst 병용 시 SFOC 최대 1.31% 개선
-  (CCS 입회 실선 엔진 시험)</t>
+  (Bio-VLSFO B30, CCS 입회 실선 엔진 시험)
+[보증 불가]</t>
         </is>
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>VLSFO : SFOC 1.454% 개선
-Bio-VLSFO (B30) : SFOC 최대 1.31% 개선
+          <t>약 1.5%
+(VLSFO, 100 ppm 조건 실측 1.454%)
+Bio-VLSFO (B30) : 최대 1.31%
 [보증 불가 — 실측 시험 자료 기준]</t>
         </is>
       </c>
@@ -1533,7 +1506,7 @@
       <c r="E29" s="9" t="inlineStr">
         <is>
           <t>HFRR 마모흔 535 µm (ULSD 단독, 부적합)
-→ 100 ppm 396 µm / 150 ppm 355 µm
+→ 100 ppm 투입 시 396 µm (합격)
 ISO 8217 (520) · EN 590 (460) 모두 충족</t>
         </is>
       </c>
@@ -1630,7 +1603,7 @@
           <t>작성 필요</t>
         </is>
       </c>
-      <c r="F32" s="12" t="inlineStr">
+      <c r="F32" s="15" t="inlineStr">
         <is>
           <t>★ 거래처별 판매실적 내부 확인 후 기입</t>
         </is>
@@ -1668,7 +1641,7 @@
 전화번호 :</t>
         </is>
       </c>
-      <c r="F33" s="12" t="inlineStr">
+      <c r="F33" s="15" t="inlineStr">
         <is>
           <t>★ 기입 필요</t>
         </is>
@@ -1681,7 +1654,7 @@
   · 노란색 셀 = 기입 필요 항목 (제품단가 / 포장 규격 / 판매실적 / 담당자 연락처 / 제품번호 · 성상 일부)
   · 파란색 숫자 = 계산 입력값. '평상시 기준 처리량'을 바꾸면 투입량과 예상 비용이 자동으로 재계산됩니다.
   · 예상 비용 = 1,000 M/T 기준 투입량 × 제품단가. 단가 입력 전에는 공란으로 표시됩니다.
-  · ★ Catalyst의 SFOC 개선 실측치(1.454% / 1.31%)는 100 ppm(1L : 10 MT) 조건에서 취득한 값입니다. 평상시 권장 투입비율(1L : 15 MT)과 다르므로, 연료절감을 제안 근거로 사용할 경우 투입량을 1L : 10 MT(1,000 M/T 당 100 L)로 산정해야 합니다.
+  · ★ Catalyst 연료절감 「약 1.5%」는 VLSFO 실측치 1.454%(100 ppm = 1L : 10 MT 조건)를 반올림한 값입니다. 본 표의 Catalyst 투입기준도 동일하게 100 ppm(1,000 M/T 당 100 L)으로 산정했습니다. Bio-VLSFO(B30)의 실측치는 최대 1.31%로 별개이며, 1.5%는 VLSFO 조건에 한합니다.
   · 본 자료의 모든 수치는 제3자 시험기관 · 선급 실측 자료에 근거하며, 연료절감률에 대한 보증은 제공되지 않습니다.</t>
         </is>
       </c>
@@ -1711,234 +1684,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="18" t="inlineStr">
-        <is>
-          <t>제품별 · 유종별 적용 범위</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="19" t="inlineStr">
-        <is>
-          <t>● 권장 (Recommended)    △ 조건부 적용 (Case by case)    –  해당 없음 (N/A)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="42" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>제품명</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>HSFO</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>VLSFO</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>Bio-VLSFO
-/ Bio-HFO
-(B30)</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>LSMGO / MGO
-/ MDO</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>Bio-LSMGO
-/ Bio-MDO</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>B100</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>기타 용도
-(Tank Mixing 등)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="20" t="inlineStr">
-        <is>
-          <t>Unitor™ FuelPower™ Conditioner</t>
-        </is>
-      </c>
-      <c r="B5" s="21" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="C5" s="21" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="D5" s="21" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="E5" s="22" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="F5" s="22" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="G5" s="22" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="H5" s="21" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="20" t="inlineStr">
-        <is>
-          <t>Unitor™ FuelPower™ Catalyst</t>
-        </is>
-      </c>
-      <c r="B6" s="21" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="C6" s="21" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="D6" s="21" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="E6" s="22" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="F6" s="22" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="G6" s="22" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="H6" s="22" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="20" t="inlineStr">
-        <is>
-          <t>Unitor™ DieselPower™ Lubricity</t>
-        </is>
-      </c>
-      <c r="B7" s="22" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C7" s="22" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="D7" s="22" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="E7" s="21" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="F7" s="23" t="inlineStr">
-        <is>
-          <t>△</t>
-        </is>
-      </c>
-      <c r="G7" s="23" t="inlineStr">
-        <is>
-          <t>△</t>
-        </is>
-      </c>
-      <c r="H7" s="22" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="96" customHeight="1">
-      <c r="A9" s="17" t="inlineStr">
-        <is>
-          <t>▣ 적용 근거 및 단서
-  · FuelPower Conditioner / Catalyst : 잔사유(Residual) 전용 제품으로 MGO 등 증류유에는 적용하지 않습니다.
-  · 기타 용도(Tank Mixing) : 서로 다른 벙커 간 혼합 시 발생하는 불호환(Incompatibility) 완화 목적의 Conditioner 적용을 의미합니다.
-  · DieselPower Lubricity — Bio-LSMGO : FAME 성분 자체가 윤활성을 보완하므로 윤활성 부적합 가능성이 낮습니다. 성적서상 HFRR 값 확인 후 적용을 판단합니다.
-  · DieselPower Lubricity — B100 : HVO(수소첨가 식물성 오일)에 한해 윤활성 저하가 나타납니다. 일반 FAME B100은 해당하지 않습니다.
-  · 본 표는 3개 제품에 한정된 것으로, 미생물 · 저온유동성 · 산화안정성 · Ash · Soot 등 그 밖의 이슈에 대해서는 별도 제품군이 적용됩니다.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A9:H9"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A1:H1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2009,94 +1754,94 @@
       </c>
     </row>
     <row r="5" ht="66" customHeight="1">
-      <c r="A5" s="24" t="n">
+      <c r="A5" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="25" t="inlineStr">
+      <c r="B5" s="20" t="inlineStr">
         <is>
           <t>Unitor™ FuelPower™ Conditioner</t>
         </is>
       </c>
-      <c r="C5" s="24" t="inlineStr">
+      <c r="C5" s="19" t="inlineStr">
         <is>
           <t>HSFO / VLSFO
 (RMG380)</t>
         </is>
       </c>
-      <c r="D5" s="26" t="inlineStr">
+      <c r="D5" s="21" t="inlineStr">
         <is>
           <t>Lloyd's Register FOBAS
 Additive Performance
 Certification Scheme</t>
         </is>
       </c>
-      <c r="E5" s="26" t="inlineStr">
+      <c r="E5" s="21" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F5" s="26" t="inlineStr">
+      <c r="F5" s="21" t="inlineStr">
         <is>
           <t>Hot Spin 침전량 평균 35.5% 감소
 (8개 항구 실측, 최고 46.67%)
 분리온도 40 / 98℃ 조건</t>
         </is>
       </c>
-      <c r="G5" s="24" t="inlineStr">
+      <c r="G5" s="19" t="inlineStr">
         <is>
           <t>Actual Trial
 (실측 시험)</t>
         </is>
       </c>
-      <c r="H5" s="26" t="inlineStr">
+      <c r="H5" s="21" t="inlineStr">
         <is>
           <t>항구별 상세 결과 하단 표 참조</t>
         </is>
       </c>
     </row>
     <row r="6" ht="66" customHeight="1">
-      <c r="A6" s="27" t="n">
+      <c r="A6" s="22" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="28" t="inlineStr">
+      <c r="B6" s="23" t="inlineStr">
         <is>
           <t>Unitor™ FuelPower™ Conditioner
 + Unitor™ FuelPower™ Catalyst</t>
         </is>
       </c>
-      <c r="C6" s="27" t="inlineStr">
+      <c r="C6" s="22" t="inlineStr">
         <is>
           <t>Bio-VLSFO (B30)
 B30 = Bio 30%,
 FAME 순도 98.8%</t>
         </is>
       </c>
-      <c r="D6" s="29" t="inlineStr">
+      <c r="D6" s="24" t="inlineStr">
         <is>
           <t>China Classification
 Society (CCS)
 Wärtsilä Letter of No Objection</t>
         </is>
       </c>
-      <c r="E6" s="29" t="inlineStr">
+      <c r="E6" s="24" t="inlineStr">
         <is>
           <t>MAN ME-C 6S35
 (Shanghai Maritime Univ.)</t>
         </is>
       </c>
-      <c r="F6" s="29" t="inlineStr">
+      <c r="F6" s="24" t="inlineStr">
         <is>
           <t>SFOC 최대 1.31% 개선
 CCS 전 구간 입회, 2초 간격 데이터 기록</t>
         </is>
       </c>
-      <c r="G6" s="27" t="inlineStr">
+      <c r="G6" s="22" t="inlineStr">
         <is>
           <t>Actual Trial
 (실측 시험)</t>
         </is>
       </c>
-      <c r="H6" s="29" t="inlineStr">
+      <c r="H6" s="24" t="inlineStr">
         <is>
           <t>CCS 검증 완료
 Hot Spin 성능은 LR 검증</t>
@@ -2104,32 +1849,32 @@
       </c>
     </row>
     <row r="7" ht="66" customHeight="1">
-      <c r="A7" s="24" t="n">
+      <c r="A7" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="25" t="inlineStr">
+      <c r="B7" s="20" t="inlineStr">
         <is>
           <t>Unitor™ FuelPower™ Catalyst</t>
         </is>
       </c>
-      <c r="C7" s="24" t="inlineStr">
+      <c r="C7" s="19" t="inlineStr">
         <is>
           <t>VLSFO</t>
         </is>
       </c>
-      <c r="D7" s="26" t="inlineStr">
+      <c r="D7" s="21" t="inlineStr">
         <is>
           <t>Veritas Petroleum
 Services (VPS)
 Wärtsilä Letter of No Objection</t>
         </is>
       </c>
-      <c r="E7" s="26" t="inlineStr">
+      <c r="E7" s="21" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F7" s="26" t="inlineStr">
+      <c r="F7" s="21" t="inlineStr">
         <is>
           <t>SFOC 1.454% 개선
 ECN (점화성 지수) 6.25% 개선
@@ -2137,13 +1882,13 @@
 (IP 541 / FIA-100 FCA 연소분석)</t>
         </is>
       </c>
-      <c r="G7" s="24" t="inlineStr">
+      <c r="G7" s="19" t="inlineStr">
         <is>
           <t>Actual Trial
 (실측 시험)</t>
         </is>
       </c>
-      <c r="H7" s="26" t="inlineStr">
+      <c r="H7" s="21" t="inlineStr">
         <is>
           <t>SFOC 시험은 Tokyo Univ. of Marine
 Science &amp; Technology 에서 고객사 실시</t>
@@ -2151,91 +1896,90 @@
       </c>
     </row>
     <row r="8" ht="66" customHeight="1">
-      <c r="A8" s="27" t="n">
+      <c r="A8" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="28" t="inlineStr">
+      <c r="B8" s="23" t="inlineStr">
         <is>
           <t>Unitor™ FuelPower™ Catalyst</t>
         </is>
       </c>
-      <c r="C8" s="27" t="inlineStr">
+      <c r="C8" s="22" t="inlineStr">
         <is>
           <t>Bio-VLSFO (B30)</t>
         </is>
       </c>
-      <c r="D8" s="29" t="inlineStr">
+      <c r="D8" s="24" t="inlineStr">
         <is>
           <t>China Classification
 Society (CCS)
 Wärtsilä Letter of No Objection</t>
         </is>
       </c>
-      <c r="E8" s="29" t="inlineStr">
+      <c r="E8" s="24" t="inlineStr">
         <is>
           <t>MAN ME-C 6S35
 (Shanghai Maritime Univ.)</t>
         </is>
       </c>
-      <c r="F8" s="29" t="inlineStr">
+      <c r="F8" s="24" t="inlineStr">
         <is>
           <t>SFOC 최대 1.31% 개선
 (Engine Trial)</t>
         </is>
       </c>
-      <c r="G8" s="27" t="inlineStr">
+      <c r="G8" s="22" t="inlineStr">
         <is>
           <t>Actual Trial
 (실측 시험)</t>
         </is>
       </c>
-      <c r="H8" s="29" t="inlineStr">
+      <c r="H8" s="24" t="inlineStr">
         <is>
           <t>CCS 검증 완료</t>
         </is>
       </c>
     </row>
     <row r="9" ht="66" customHeight="1">
-      <c r="A9" s="24" t="n">
+      <c r="A9" s="19" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="25" t="inlineStr">
+      <c r="B9" s="20" t="inlineStr">
         <is>
           <t>Unitor™ DieselPower™ Lubricity</t>
         </is>
       </c>
-      <c r="C9" s="24" t="inlineStr">
+      <c r="C9" s="19" t="inlineStr">
         <is>
           <t>LSMGO / ULSD</t>
         </is>
       </c>
-      <c r="D9" s="26" t="inlineStr">
+      <c r="D9" s="21" t="inlineStr">
         <is>
           <t>Lloyd's Register
 Product Verification Scheme
 ISO 12156-1 (HFRR)</t>
         </is>
       </c>
-      <c r="E9" s="26" t="inlineStr">
+      <c r="E9" s="21" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F9" s="26" t="inlineStr">
+      <c r="F9" s="21" t="inlineStr">
         <is>
           <t>HFRR 마모흔 (WS1.4, µm)
 · ULSD 단독 : 535 (부적합)
-· + 100 ppm : 396 (합격)
-· + 150 ppm : 355 (합격)</t>
-        </is>
-      </c>
-      <c r="G9" s="24" t="inlineStr">
+· + 100 ppm (1L : 10 MT) : 396 (합격)</t>
+        </is>
+      </c>
+      <c r="G9" s="19" t="inlineStr">
         <is>
           <t>Lab Test
 (사내 시험)</t>
         </is>
       </c>
-      <c r="H9" s="26" t="inlineStr">
+      <c r="H9" s="21" t="inlineStr">
         <is>
           <t>ISO 8217 한계 520 µm,
 EN 590 한계 460 µm 모두 충족</t>
@@ -2243,310 +1987,310 @@
       </c>
     </row>
     <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="30" t="inlineStr">
+      <c r="A11" s="25" t="inlineStr">
         <is>
           <t>[상세] Unitor™ FuelPower™ Conditioner — Hot Spin Test 항구별 실측 결과 (RMG380)</t>
         </is>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1">
-      <c r="A12" s="31" t="inlineStr">
+      <c r="A12" s="26" t="inlineStr">
         <is>
           <t>항구</t>
         </is>
       </c>
-      <c r="B12" s="31" t="inlineStr">
+      <c r="B12" s="26" t="inlineStr">
         <is>
           <t>점도
 (cSt @50℃)</t>
         </is>
       </c>
-      <c r="C12" s="31" t="inlineStr">
+      <c r="C12" s="26" t="inlineStr">
         <is>
           <t>MCR (%)</t>
         </is>
       </c>
-      <c r="D12" s="31" t="inlineStr">
+      <c r="D12" s="26" t="inlineStr">
         <is>
           <t>분리온도
 (℃)</t>
         </is>
       </c>
-      <c r="E12" s="31" t="inlineStr">
+      <c r="E12" s="26" t="inlineStr">
         <is>
           <t>Before
 (침전 %)</t>
         </is>
       </c>
-      <c r="F12" s="31" t="inlineStr">
+      <c r="F12" s="26" t="inlineStr">
         <is>
           <t>After
 (침전 %)</t>
         </is>
       </c>
-      <c r="G12" s="31" t="inlineStr">
+      <c r="G12" s="26" t="inlineStr">
         <is>
           <t>개선율 (%)</t>
         </is>
       </c>
-      <c r="H12" s="31" t="inlineStr">
+      <c r="H12" s="26" t="inlineStr">
         <is>
           <t>비고</t>
         </is>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="32" t="inlineStr">
+      <c r="A13" s="27" t="inlineStr">
         <is>
           <t>Zeebrugge</t>
         </is>
       </c>
-      <c r="B13" s="33" t="n">
+      <c r="B13" s="28" t="n">
         <v>335.2</v>
       </c>
-      <c r="C13" s="34" t="n">
+      <c r="C13" s="29" t="n">
         <v>11.6</v>
       </c>
-      <c r="D13" s="35" t="n">
+      <c r="D13" s="30" t="n">
         <v>98</v>
       </c>
-      <c r="E13" s="34" t="n">
+      <c r="E13" s="29" t="n">
         <v>0.19</v>
       </c>
-      <c r="F13" s="34" t="n">
+      <c r="F13" s="29" t="n">
         <v>0.13</v>
       </c>
-      <c r="G13" s="36">
+      <c r="G13" s="31">
         <f>(E13-F13)/E13</f>
         <v/>
       </c>
-      <c r="H13" s="37" t="inlineStr"/>
+      <c r="H13" s="32" t="inlineStr"/>
     </row>
     <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="32" t="inlineStr">
+      <c r="A14" s="27" t="inlineStr">
         <is>
           <t>Tuapse</t>
         </is>
       </c>
-      <c r="B14" s="33" t="n">
+      <c r="B14" s="28" t="n">
         <v>18.9</v>
       </c>
-      <c r="C14" s="34" t="n">
+      <c r="C14" s="29" t="n">
         <v>2.96</v>
       </c>
-      <c r="D14" s="35" t="n">
+      <c r="D14" s="30" t="n">
         <v>40</v>
       </c>
-      <c r="E14" s="34" t="n">
+      <c r="E14" s="29" t="n">
         <v>0.24</v>
       </c>
-      <c r="F14" s="34" t="n">
+      <c r="F14" s="29" t="n">
         <v>0.2</v>
       </c>
-      <c r="G14" s="36">
+      <c r="G14" s="31">
         <f>(E14-F14)/E14</f>
         <v/>
       </c>
-      <c r="H14" s="37" t="inlineStr">
+      <c r="H14" s="32" t="inlineStr">
         <is>
           <t>저점도 · 분리온도 40℃ 조건</t>
         </is>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="32" t="inlineStr">
+      <c r="A15" s="27" t="inlineStr">
         <is>
           <t>Amsterdam</t>
         </is>
       </c>
-      <c r="B15" s="33" t="n">
+      <c r="B15" s="28" t="n">
         <v>206.6</v>
       </c>
-      <c r="C15" s="34" t="n">
+      <c r="C15" s="29" t="n">
         <v>10.91</v>
       </c>
-      <c r="D15" s="35" t="n">
+      <c r="D15" s="30" t="n">
         <v>98</v>
       </c>
-      <c r="E15" s="34" t="n">
+      <c r="E15" s="29" t="n">
         <v>0.15</v>
       </c>
-      <c r="F15" s="34" t="n">
+      <c r="F15" s="29" t="n">
         <v>0.08</v>
       </c>
-      <c r="G15" s="36">
+      <c r="G15" s="31">
         <f>(E15-F15)/E15</f>
         <v/>
       </c>
-      <c r="H15" s="37" t="inlineStr"/>
+      <c r="H15" s="32" t="inlineStr"/>
     </row>
     <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="32" t="inlineStr">
+      <c r="A16" s="27" t="inlineStr">
         <is>
           <t>Flushing</t>
         </is>
       </c>
-      <c r="B16" s="33" t="n">
+      <c r="B16" s="28" t="n">
         <v>239.7</v>
       </c>
-      <c r="C16" s="34" t="n">
+      <c r="C16" s="29" t="n">
         <v>9.08</v>
       </c>
-      <c r="D16" s="35" t="n">
+      <c r="D16" s="30" t="n">
         <v>98</v>
       </c>
-      <c r="E16" s="34" t="n">
+      <c r="E16" s="29" t="n">
         <v>0.13</v>
       </c>
-      <c r="F16" s="34" t="n">
+      <c r="F16" s="29" t="n">
         <v>0.09</v>
       </c>
-      <c r="G16" s="36">
+      <c r="G16" s="31">
         <f>(E16-F16)/E16</f>
         <v/>
       </c>
-      <c r="H16" s="37" t="inlineStr"/>
+      <c r="H16" s="32" t="inlineStr"/>
     </row>
     <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="32" t="inlineStr">
+      <c r="A17" s="27" t="inlineStr">
         <is>
           <t>Duqm</t>
         </is>
       </c>
-      <c r="B17" s="33" t="n">
+      <c r="B17" s="28" t="n">
         <v>230.7</v>
       </c>
-      <c r="C17" s="34" t="n">
+      <c r="C17" s="29" t="n">
         <v>7.15</v>
       </c>
-      <c r="D17" s="35" t="n">
+      <c r="D17" s="30" t="n">
         <v>98</v>
       </c>
-      <c r="E17" s="34" t="n">
+      <c r="E17" s="29" t="n">
         <v>0.33</v>
       </c>
-      <c r="F17" s="34" t="n">
+      <c r="F17" s="29" t="n">
         <v>0.2</v>
       </c>
-      <c r="G17" s="36">
+      <c r="G17" s="31">
         <f>(E17-F17)/E17</f>
         <v/>
       </c>
-      <c r="H17" s="37" t="inlineStr"/>
+      <c r="H17" s="32" t="inlineStr"/>
     </row>
     <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="32" t="inlineStr">
+      <c r="A18" s="27" t="inlineStr">
         <is>
           <t>Amsterdam</t>
         </is>
       </c>
-      <c r="B18" s="33" t="n">
+      <c r="B18" s="28" t="n">
         <v>314.4</v>
       </c>
-      <c r="C18" s="34" t="n">
+      <c r="C18" s="29" t="n">
         <v>10.02</v>
       </c>
-      <c r="D18" s="35" t="n">
+      <c r="D18" s="30" t="n">
         <v>98</v>
       </c>
-      <c r="E18" s="34" t="n">
+      <c r="E18" s="29" t="n">
         <v>0.16</v>
       </c>
-      <c r="F18" s="34" t="n">
+      <c r="F18" s="29" t="n">
         <v>0.1</v>
       </c>
-      <c r="G18" s="36">
+      <c r="G18" s="31">
         <f>(E18-F18)/E18</f>
         <v/>
       </c>
-      <c r="H18" s="37" t="inlineStr"/>
+      <c r="H18" s="32" t="inlineStr"/>
     </row>
     <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="32" t="inlineStr">
+      <c r="A19" s="27" t="inlineStr">
         <is>
           <t>Vlissingen</t>
         </is>
       </c>
-      <c r="B19" s="33" t="n">
+      <c r="B19" s="28" t="n">
         <v>242.8</v>
       </c>
-      <c r="C19" s="34" t="n">
+      <c r="C19" s="29" t="n">
         <v>10.5</v>
       </c>
-      <c r="D19" s="35" t="n">
+      <c r="D19" s="30" t="n">
         <v>98</v>
       </c>
-      <c r="E19" s="34" t="n">
+      <c r="E19" s="29" t="n">
         <v>0.13</v>
       </c>
-      <c r="F19" s="34" t="n">
+      <c r="F19" s="29" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="G19" s="36">
+      <c r="G19" s="31">
         <f>(E19-F19)/E19</f>
         <v/>
       </c>
-      <c r="H19" s="37" t="inlineStr"/>
+      <c r="H19" s="32" t="inlineStr"/>
     </row>
     <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="32" t="inlineStr">
+      <c r="A20" s="27" t="inlineStr">
         <is>
           <t>Callao</t>
         </is>
       </c>
-      <c r="B20" s="33" t="n">
+      <c r="B20" s="28" t="n">
         <v>335.1</v>
       </c>
-      <c r="C20" s="34" t="n">
+      <c r="C20" s="29" t="n">
         <v>8.84</v>
       </c>
-      <c r="D20" s="35" t="n">
+      <c r="D20" s="30" t="n">
         <v>98</v>
       </c>
-      <c r="E20" s="34" t="n">
+      <c r="E20" s="29" t="n">
         <v>0.17</v>
       </c>
-      <c r="F20" s="34" t="n">
+      <c r="F20" s="29" t="n">
         <v>0.11</v>
       </c>
-      <c r="G20" s="36">
+      <c r="G20" s="31">
         <f>(E20-F20)/E20</f>
         <v/>
       </c>
-      <c r="H20" s="37" t="inlineStr"/>
+      <c r="H20" s="32" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="31" t="inlineStr">
+      <c r="A21" s="26" t="inlineStr">
         <is>
           <t>평균</t>
         </is>
       </c>
-      <c r="B21" s="38">
+      <c r="B21" s="33">
         <f>AVERAGE(B13:B20)</f>
         <v/>
       </c>
-      <c r="C21" s="38">
+      <c r="C21" s="33">
         <f>AVERAGE(C13:C20)</f>
         <v/>
       </c>
-      <c r="D21" s="31" t="inlineStr">
+      <c r="D21" s="26" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E21" s="38">
+      <c r="E21" s="33">
         <f>AVERAGE(E13:E20)</f>
         <v/>
       </c>
-      <c r="F21" s="38">
+      <c r="F21" s="33">
         <f>AVERAGE(F13:F20)</f>
         <v/>
       </c>
-      <c r="G21" s="39">
+      <c r="G21" s="34">
         <f>AVERAGE(G13:G20)</f>
         <v/>
       </c>
-      <c r="H21" s="40" t="inlineStr">
+      <c r="H21" s="35" t="inlineStr">
         <is>
           <t>최고 개선율 46.67% (Amsterdam)</t>
         </is>
@@ -2574,13 +2318,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2607,15 +2351,15 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="41" t="inlineStr">
+      <c r="A4" s="36" t="inlineStr">
         <is>
           <t>벙커량 (M/T)</t>
         </is>
       </c>
-      <c r="B4" s="42" t="n">
+      <c r="B4" s="37" t="n">
         <v>1000</v>
       </c>
-      <c r="C4" s="43" t="inlineStr">
+      <c r="C4" s="38" t="inlineStr">
         <is>
           <t>← 실제 벙커 수량을 입력하십시오 (기본값 1,000 M/T)</t>
         </is>
@@ -2661,228 +2405,207 @@
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="20" t="inlineStr">
+      <c r="A7" s="39" t="inlineStr">
         <is>
           <t>Unitor™ FuelPower™ Conditioner</t>
         </is>
       </c>
-      <c r="B7" s="27" t="inlineStr">
+      <c r="B7" s="22" t="inlineStr">
         <is>
           <t>HSFO / VLSFO /
 Bio-VLSFO</t>
         </is>
       </c>
-      <c r="C7" s="29" t="inlineStr">
+      <c r="C7" s="24" t="inlineStr">
         <is>
           <t>평상시 (General)</t>
         </is>
       </c>
-      <c r="D7" s="13" t="n">
+      <c r="D7" s="12" t="n">
         <v>15</v>
       </c>
-      <c r="E7" s="14">
+      <c r="E7" s="13">
         <f>ROUND($B$4/D7,0)</f>
         <v/>
       </c>
-      <c r="F7" s="15" t="n"/>
+      <c r="F7" s="14" t="n"/>
       <c r="G7" s="16">
         <f>IF(F7="","",E7*F7)</f>
         <v/>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="44" t="n"/>
-      <c r="B8" s="44" t="n"/>
-      <c r="C8" s="29" t="inlineStr">
+      <c r="A8" s="40" t="n"/>
+      <c r="B8" s="40" t="n"/>
+      <c r="C8" s="24" t="inlineStr">
         <is>
           <t>최대 (Max.)</t>
         </is>
       </c>
-      <c r="D8" s="13" t="n">
+      <c r="D8" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="E8" s="14">
+      <c r="E8" s="13">
         <f>ROUND($B$4/D8,0)</f>
         <v/>
       </c>
-      <c r="F8" s="15" t="n"/>
+      <c r="F8" s="14" t="n"/>
       <c r="G8" s="16">
         <f>IF(F8="","",E8*F8)</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="45" t="n"/>
-      <c r="B9" s="45" t="n"/>
-      <c r="C9" s="29" t="inlineStr">
+      <c r="A9" s="41" t="n"/>
+      <c r="B9" s="41" t="n"/>
+      <c r="C9" s="24" t="inlineStr">
         <is>
           <t>최소 (Min.)</t>
         </is>
       </c>
-      <c r="D9" s="13" t="n">
+      <c r="D9" s="12" t="n">
         <v>25</v>
       </c>
-      <c r="E9" s="14">
+      <c r="E9" s="13">
         <f>ROUND($B$4/D9,0)</f>
         <v/>
       </c>
-      <c r="F9" s="15" t="n"/>
+      <c r="F9" s="14" t="n"/>
       <c r="G9" s="16">
         <f>IF(F9="","",E9*F9)</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="20" t="inlineStr">
+      <c r="A10" s="39" t="inlineStr">
         <is>
           <t>Unitor™ FuelPower™ Catalyst</t>
         </is>
       </c>
-      <c r="B10" s="27" t="inlineStr">
+      <c r="B10" s="22" t="inlineStr">
         <is>
           <t>HSFO / VLSFO /
 Bio-VLSFO</t>
         </is>
       </c>
-      <c r="C10" s="29" t="inlineStr">
-        <is>
-          <t>평상시 (General)</t>
-        </is>
-      </c>
-      <c r="D10" s="13" t="n">
-        <v>15</v>
-      </c>
-      <c r="E10" s="14">
+      <c r="C10" s="15" t="inlineStr">
+        <is>
+          <t>★ 평상시 · 연료절감 실측 조건 (100 ppm)</t>
+        </is>
+      </c>
+      <c r="D10" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="E10" s="13">
         <f>ROUND($B$4/D10,0)</f>
         <v/>
       </c>
-      <c r="F10" s="15" t="n"/>
+      <c r="F10" s="14" t="n"/>
       <c r="G10" s="16">
         <f>IF(F10="","",E10*F10)</f>
         <v/>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="44" t="n"/>
-      <c r="B11" s="44" t="n"/>
-      <c r="C11" s="12" t="inlineStr">
-        <is>
-          <t>★ 연료절감 실측 조건 (100 ppm)</t>
-        </is>
-      </c>
-      <c r="D11" s="13" t="n">
-        <v>10</v>
-      </c>
-      <c r="E11" s="14">
+      <c r="A11" s="40" t="n"/>
+      <c r="B11" s="40" t="n"/>
+      <c r="C11" s="24" t="inlineStr">
+        <is>
+          <t>제품 사양상 General</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="n">
+        <v>15</v>
+      </c>
+      <c r="E11" s="13">
         <f>ROUND($B$4/D11,0)</f>
         <v/>
       </c>
-      <c r="F11" s="15" t="n"/>
+      <c r="F11" s="14" t="n"/>
       <c r="G11" s="16">
         <f>IF(F11="","",E11*F11)</f>
         <v/>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="45" t="n"/>
-      <c r="B12" s="45" t="n"/>
-      <c r="C12" s="29" t="inlineStr">
+      <c r="A12" s="41" t="n"/>
+      <c r="B12" s="41" t="n"/>
+      <c r="C12" s="24" t="inlineStr">
         <is>
           <t>최대 (Max.)</t>
         </is>
       </c>
-      <c r="D12" s="13" t="n">
+      <c r="D12" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="E12" s="14">
+      <c r="E12" s="13">
         <f>ROUND($B$4/D12,0)</f>
         <v/>
       </c>
-      <c r="F12" s="15" t="n"/>
+      <c r="F12" s="14" t="n"/>
       <c r="G12" s="16">
         <f>IF(F12="","",E12*F12)</f>
         <v/>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="20" t="inlineStr">
+      <c r="A13" s="39" t="inlineStr">
         <is>
           <t>Unitor™ DieselPower™ Lubricity</t>
         </is>
       </c>
-      <c r="B13" s="27" t="inlineStr">
+      <c r="B13" s="22" t="inlineStr">
         <is>
           <t>LSMGO / MGO /
 MDO</t>
         </is>
       </c>
-      <c r="C13" s="29" t="inlineStr">
-        <is>
-          <t>평상시 (General, 100 ppm)</t>
-        </is>
-      </c>
-      <c r="D13" s="13" t="n">
+      <c r="C13" s="15" t="inlineStr">
+        <is>
+          <t>★ 평상시 (100 ppm) — HFRR 396 µm</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="n">
         <v>10</v>
       </c>
-      <c r="E13" s="14">
+      <c r="E13" s="13">
         <f>ROUND($B$4/D13,0)</f>
         <v/>
       </c>
-      <c r="F13" s="15" t="n"/>
+      <c r="F13" s="14" t="n"/>
       <c r="G13" s="16">
         <f>IF(F13="","",E13*F13)</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="44" t="n"/>
-      <c r="B14" s="44" t="n"/>
-      <c r="C14" s="29" t="inlineStr">
-        <is>
-          <t>시험 근거 (125 ppm)</t>
-        </is>
-      </c>
-      <c r="D14" s="13" t="n">
-        <v>8</v>
-      </c>
-      <c r="E14" s="14">
+      <c r="A14" s="41" t="n"/>
+      <c r="B14" s="41" t="n"/>
+      <c r="C14" s="24" t="inlineStr">
+        <is>
+          <t>최대 (Max., 200 ppm)</t>
+        </is>
+      </c>
+      <c r="D14" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="E14" s="13">
         <f>ROUND($B$4/D14,0)</f>
         <v/>
       </c>
-      <c r="F14" s="15" t="n"/>
+      <c r="F14" s="14" t="n"/>
       <c r="G14" s="16">
         <f>IF(F14="","",E14*F14)</f>
         <v/>
       </c>
     </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="45" t="n"/>
-      <c r="B15" s="45" t="n"/>
-      <c r="C15" s="29" t="inlineStr">
-        <is>
-          <t>최대 (Max., 200 ppm)</t>
-        </is>
-      </c>
-      <c r="D15" s="13" t="n">
-        <v>5</v>
-      </c>
-      <c r="E15" s="14">
-        <f>ROUND($B$4/D15,0)</f>
-        <v/>
-      </c>
-      <c r="F15" s="15" t="n"/>
-      <c r="G15" s="16">
-        <f>IF(F15="","",E15*F15)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17" ht="90" customHeight="1">
-      <c r="A17" s="17" t="inlineStr">
+    <row r="16" ht="90" customHeight="1">
+      <c r="A16" s="17" t="inlineStr">
         <is>
           <t>▣ 산출 기준
   · 필요 투입량 (L) = 벙커량 (M/T) ÷ 투입 비율 (1 L 당 처리 MT), 리터 단위 반올림
   · 예상 비용 (USD) = 필요 투입량 × 제품단가. 단가 입력 전에는 공란으로 표시됩니다.
-  · ★ FuelPower Catalyst 의 SFOC 개선 실측치(VLSFO 1.454% / Bio-VLSFO 1.31%)는 100 ppm(1L : 10 MT) 조건에서 취득한 값입니다. 연료절감을 근거로 제안할 경우 이 행을 기준으로 산출하십시오.
+  · ★ 표시 행이 제안 기준입니다. FuelPower Catalyst 의 연료절감 「약 1.5%」(VLSFO 실측 1.454%)와 DieselPower Lubricity 의 HFRR 396 µm 는 모두 100 ppm(1L : 10 MT) 조건에서 취득한 값이므로, 이 행을 기준으로 산출하십시오.
   · Conditioner 와 Catalyst 를 병용할 경우 두 제품의 투입량과 비용을 각각 합산해야 합니다. (Bio-VLSFO B30 실선 시험은 Catalyst 1L + Conditioner 1L per 10 MT 조건에서 수행되었습니다.)</t>
         </is>
       </c>
@@ -2892,13 +2615,13 @@
     <mergeCell ref="C4:G4"/>
     <mergeCell ref="A7:A9"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A17:G17"/>
     <mergeCell ref="B10:B12"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="B13:B14"/>
     <mergeCell ref="A10:A12"/>
-    <mergeCell ref="B13:B15"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="B7:B9"/>
-    <mergeCell ref="A13:A15"/>
+    <mergeCell ref="A16:G16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>